<commit_message>
Added mixed integer and linear optimization
</commit_message>
<xml_diff>
--- a/docs/examples/00-overview.xlsx
+++ b/docs/examples/00-overview.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>cvxx: Convex Optimization in Excel</t>
   </si>
@@ -74,6 +74,12 @@
   </si>
   <si>
     <t>Re-examining a solved diet problem: reading back status, cost, quantities, and handle descriptions.</t>
+  </si>
+  <si>
+    <t>08-mixed-integer-programming.xlsx</t>
+  </si>
+  <si>
+    <t>Project selection: choosing which proposals to fund (yes/no decisions) within a fixed budget.</t>
   </si>
 </sst>
 </file>
@@ -464,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
@@ -608,8 +614,20 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
@@ -622,6 +640,7 @@
     <mergeCell ref="B11:F11"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>